<commit_message>
This represents Discovery and Extract stages completed. The scripts and testing were completed for both Discovery and Extraction.
</commit_message>
<xml_diff>
--- a/docs/ChatGPT Upload Docs/AlphaOmega Data Dictionary.xlsx
+++ b/docs/ChatGPT Upload Docs/AlphaOmega Data Dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/70ee5aa1d6a4da1f/AlphaOmega/Docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/70ee5aa1d6a4da1f/AlphaOmega/docs/ChatGPT Upload Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="92" documentId="8_{EEE9038B-07F8-4E74-ABBD-DCE8BEFA068C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2AEB67D0-3371-40F0-9EDB-80BD8EE11132}"/>
+  <xr:revisionPtr revIDLastSave="100" documentId="8_{EEE9038B-07F8-4E74-ABBD-DCE8BEFA068C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B72FDB1B-1BD0-454E-857A-47CA4F0BB214}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{2E56D5ED-1CE4-4881-8D7B-73E549022760}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{2E56D5ED-1CE4-4881-8D7B-73E549022760}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="1" r:id="rId1"/>
@@ -176,18 +176,12 @@
     <t>source_path</t>
   </si>
   <si>
-    <t>Human-readable source location.</t>
-  </si>
-  <si>
     <t>source_url</t>
   </si>
   <si>
     <t>title</t>
   </si>
   <si>
-    <t>Canonical title.</t>
-  </si>
-  <si>
     <t>object_type</t>
   </si>
   <si>
@@ -198,9 +192,6 @@
   </si>
   <si>
     <t>content_hash</t>
-  </si>
-  <si>
-    <t>Detects meaningful content changes.</t>
   </si>
   <si>
     <t>source_created_at</t>
@@ -391,12 +382,6 @@
     <t>External Identifier</t>
   </si>
   <si>
-    <t>Original object ID from the source.</t>
-  </si>
-  <si>
-    <t>Parent object identifier.</t>
-  </si>
-  <si>
     <t>Path</t>
   </si>
   <si>
@@ -412,9 +397,6 @@
     <t>Hash</t>
   </si>
   <si>
-    <t>Last modification timestamp from the source.</t>
-  </si>
-  <si>
     <t>Source-specific metadata.</t>
   </si>
   <si>
@@ -469,9 +451,6 @@
     <t>Job created because of the event.</t>
   </si>
   <si>
-    <t>Created, Modified, Deleted, Renamed, etc.</t>
-  </si>
-  <si>
     <t>Source-reported modification time.</t>
   </si>
   <si>
@@ -509,6 +488,27 @@
   </si>
   <si>
     <t>domain_id</t>
+  </si>
+  <si>
+    <t>Stable object identifier assigned by the Source of Truth. Combined with source_id to identify the corresponding source object during synchronization and preserve traceability.</t>
+  </si>
+  <si>
+    <t>Immediate parent object identifier assigned by the Source of Truth. Used by Discovery to detect when an existing source object has moved.</t>
+  </si>
+  <si>
+    <t>Human-readable source ancestry retained for traceability, diagnostics, and source context. Not used by Discovery for object identity or change detection.</t>
+  </si>
+  <si>
+    <t>Canonical source object name persisted by AlphaOmega. Compared by Discovery to detect when an existing source object has been renamed.</t>
+  </si>
+  <si>
+    <t>Hash of canonical content generated by Extraction and persisted for canonical content integrity and downstream comparison needs. Not used by Discovery to determine synchronization state.</t>
+  </si>
+  <si>
+    <t>Last modification timestamp reported by the Source of Truth. Compared by Discovery when determining whether an existing source object has been modified.</t>
+  </si>
+  <si>
+    <t>Synchronization state observed by Discovery: New or Modified. Additional change details, such as rename or move, may be preserved in metadata.</t>
   </si>
 </sst>
 </file>
@@ -595,9 +595,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -611,6 +608,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -982,7 +982,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -990,7 +990,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1018,10 +1018,10 @@
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B10" s="3"/>
+      <c r="A10" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1037,24 +1037,24 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="61.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="45.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="61.85546875" style="5"/>
+    <col min="1" max="1" width="11.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="45.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="61.85546875" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>14</v>
@@ -1071,9 +1071,9 @@
         <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C2" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -1083,7 +1083,7 @@
         <v>20</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1091,9 +1091,9 @@
         <v>21</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C3" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="2" t="s">
@@ -1111,19 +1111,19 @@
         <v>24</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C4" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1131,9 +1131,9 @@
         <v>25</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C5" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="2" t="s">
@@ -1143,7 +1143,7 @@
         <v>19</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1151,9 +1151,9 @@
         <v>26</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C6" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>27</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -1163,7 +1163,7 @@
         <v>19</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1171,9 +1171,9 @@
         <v>28</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C7" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D7" s="2" t="s">
@@ -1183,7 +1183,7 @@
         <v>20</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1191,9 +1191,9 @@
         <v>30</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C8" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D8" s="2" t="s">
@@ -1203,7 +1203,7 @@
         <v>19</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1211,19 +1211,19 @@
         <v>31</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1231,9 +1231,9 @@
         <v>32</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C10" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>33</v>
       </c>
       <c r="D10" s="2" t="s">
@@ -1243,7 +1243,7 @@
         <v>19</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1257,24 +1257,24 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="35.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.85546875" style="5" customWidth="1"/>
-    <col min="7" max="16384" width="35.140625" style="5"/>
+    <col min="1" max="1" width="17.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.85546875" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="35.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>14</v>
@@ -1291,9 +1291,9 @@
         <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C2" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -1303,17 +1303,17 @@
         <v>20</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="2" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C3" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D3" s="2" t="s">
@@ -1323,7 +1323,7 @@
         <v>19</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1331,9 +1331,9 @@
         <v>21</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
@@ -1343,7 +1343,7 @@
         <v>19</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1351,9 +1351,9 @@
         <v>25</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C5" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="2" t="s">
@@ -1363,7 +1363,7 @@
         <v>19</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1371,9 +1371,9 @@
         <v>34</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C6" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -1383,17 +1383,17 @@
         <v>19</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="2" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C7" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="2" t="s">
@@ -1411,9 +1411,9 @@
         <v>36</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C8" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="2" t="s">
@@ -1423,7 +1423,7 @@
         <v>19</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1431,9 +1431,9 @@
         <v>28</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C9" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
@@ -1443,7 +1443,7 @@
         <v>20</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1451,9 +1451,9 @@
         <v>30</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C10" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D10" s="2" t="s">
@@ -1463,7 +1463,7 @@
         <v>19</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1471,9 +1471,9 @@
         <v>32</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C11" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>33</v>
       </c>
       <c r="D11" s="2" t="s">
@@ -1483,7 +1483,7 @@
         <v>19</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1497,24 +1497,24 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultColWidth="42" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="42" style="5"/>
+    <col min="1" max="1" width="22.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="42" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>14</v>
@@ -1531,9 +1531,9 @@
         <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C2" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -1543,7 +1543,7 @@
         <v>20</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1551,9 +1551,9 @@
         <v>37</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D3" s="2" t="s">
@@ -1563,17 +1563,17 @@
         <v>20</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="2" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
@@ -1583,37 +1583,37 @@
         <v>19</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="75">
       <c r="A5" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C5" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="60">
       <c r="A6" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C6" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -1623,17 +1623,17 @@
         <v>19</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="60">
       <c r="A7" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C7" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="2" t="s">
@@ -1643,39 +1643,39 @@
         <v>19</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>41</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="60">
+      <c r="A9" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C8" s="6" t="s">
+      <c r="B9" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="D9" s="2" t="s">
         <v>19</v>
       </c>
@@ -1683,17 +1683,17 @@
         <v>19</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>44</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C10" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="2" t="s">
@@ -1703,17 +1703,17 @@
         <v>19</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C11" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D11" s="2" t="s">
@@ -1723,17 +1723,17 @@
         <v>19</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="75">
       <c r="A12" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C12" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D12" s="2" t="s">
@@ -1743,17 +1743,17 @@
         <v>19</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>49</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C13" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D13" s="2" t="s">
@@ -1763,17 +1763,17 @@
         <v>19</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="60">
       <c r="A14" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C14" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D14" s="2" t="s">
@@ -1783,17 +1783,17 @@
         <v>19</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>102</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C15" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D15" s="2" t="s">
@@ -1803,7 +1803,7 @@
         <v>20</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1811,9 +1811,9 @@
         <v>32</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C16" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>33</v>
       </c>
       <c r="D16" s="2" t="s">
@@ -1823,7 +1823,7 @@
         <v>19</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1837,24 +1837,24 @@
   <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="23.5703125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.5703125" style="5"/>
-    <col min="3" max="3" width="18.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="23.5703125" style="5"/>
+    <col min="1" max="1" width="19.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5703125" style="4"/>
+    <col min="3" max="3" width="18.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="23.5703125" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>14</v>
@@ -1871,9 +1871,9 @@
         <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C2" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -1883,17 +1883,17 @@
         <v>20</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D3" s="2" t="s">
@@ -1903,7 +1903,7 @@
         <v>20</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1911,9 +1911,9 @@
         <v>37</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
@@ -1923,17 +1923,17 @@
         <v>20</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="2" t="s">
@@ -1943,17 +1943,17 @@
         <v>20</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C6" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -1963,37 +1963,37 @@
         <v>20</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C7" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C8" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D8" s="2" t="s">
@@ -2003,57 +2003,57 @@
         <v>20</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C9" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C10" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C11" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D11" s="2" t="s">
@@ -2063,7 +2063,7 @@
         <v>20</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2071,19 +2071,19 @@
         <v>32</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C12" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>33</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2097,24 +2097,24 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.42578125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="22.28515625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="20.42578125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="22.28515625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>14</v>
@@ -2127,163 +2127,163 @@
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="60">
+      <c r="A6" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="7" t="s">
+      <c r="C6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="C7" s="8" t="s">
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>122</v>
+      <c r="D8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="C9" s="8" t="s">
+      <c r="B9" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>123</v>
+      <c r="D9" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>